<commit_message>
SORT_DATA 자동 동기화: SCRAPPIESといっしょ 신규 리뷰 추가 (#76, SCRAP - Mystery For You)
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/검색어_맵핑.xlsx
+++ b/검색어_맵핑.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1634,26 +1634,21 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n"/>
-      <c r="B69" s="2" t="n"/>
-      <c r="C69" s="2" t="n"/>
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>SCRAPPIESといっしょ</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>tumbleweed</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>텀블위드, 탐블위도, 탐블위드</t>
-        </is>
-      </c>
+      <c r="A70" s="2" t="n"/>
+      <c r="B70" s="2" t="n"/>
+      <c r="C70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -1663,12 +1658,12 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>키이스케이프</t>
+          <t>tumbleweed</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>keyescape</t>
+          <t>텀블위드, 탐블위도, 탐블위드</t>
         </is>
       </c>
     </row>
@@ -1680,12 +1675,12 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>NAZOxNAZO劇団</t>
-        </is>
-      </c>
-      <c r="C72" s="4" t="inlineStr">
-        <is>
-          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
+          <t>키이스케이프</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>keyescape</t>
         </is>
       </c>
     </row>
@@ -1697,12 +1692,12 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>MICHI</t>
-        </is>
-      </c>
-      <c r="C73" s="3" t="inlineStr">
-        <is>
-          <t>미치</t>
+          <t>NAZOxNAZO劇団</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>나조x나조극단, 나조x나조 극단, 나조나조극단, 나조x나조게키단, 나조나조게키단,나조,극단,게키단</t>
         </is>
       </c>
     </row>
@@ -1714,12 +1709,12 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>ぐずりあ</t>
+          <t>MICHI</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>구스리아</t>
+          <t>미치</t>
         </is>
       </c>
     </row>
@@ -1731,12 +1726,12 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>時解き</t>
+          <t>ぐずりあ</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>토키토키, tokitoki,토키,toki</t>
+          <t>구스리아</t>
         </is>
       </c>
     </row>
@@ -1748,12 +1743,12 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Mystery Lunch</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="inlineStr">
-        <is>
-          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+          <t>時解き</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>토키토키, tokitoki,토키,toki</t>
         </is>
       </c>
     </row>
@@ -1765,29 +1760,29 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
+          <t>Mystery Lunch</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>미스테리 런치, 미스터리 런치, 미스테리런치, 미스터리런치,미스터리,미스테리,런치,점심</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
           <t>SCRAP</t>
         </is>
       </c>
-      <c r="C77" s="3" t="inlineStr">
+      <c r="C78" s="3" t="inlineStr">
         <is>
           <t>스크랩, 스크랍뿌, 스크랍부, 스크랏푸, 스크랏뿌, 스크렙</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>브랜드</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>SCRAP - Mystery For You</t>
-        </is>
-      </c>
-      <c r="C78" s="8" t="inlineStr">
-        <is>
-          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
         </is>
       </c>
     </row>
@@ -1799,12 +1794,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>4CE Dimension</t>
+          <t>SCRAP - Mystery For You</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>포스 디멘션, 포스 디멘젼</t>
+          <t>스크랩 - 미스터리 포유, 미스터리 포유, 미포유, Mystery For You, MFY</t>
         </is>
       </c>
     </row>
@@ -1816,12 +1811,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>AnotherVision</t>
+          <t>4CE Dimension</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t>어나더비젼, 어나더비전, 어나더 비전, 어나더 비젼, 도쿄대 걔네</t>
+          <t>포스 디멘션, 포스 디멘젼</t>
         </is>
       </c>
     </row>
@@ -1833,12 +1828,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>xeoxy</t>
+          <t>AnotherVision</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>제옥시</t>
+          <t>어나더비젼, 어나더비전, 어나더 비전, 어나더 비젼, 도쿄대 걔네</t>
         </is>
       </c>
     </row>
@@ -1850,12 +1845,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>リドラ</t>
+          <t>xeoxy</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t>리도라, 리들러</t>
+          <t>제옥시</t>
         </is>
       </c>
     </row>
@@ -1867,29 +1862,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ねずみの巣</t>
+          <t>リドラ</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t>쥐의굴, 쥐의 굴, 네즈미노 스, 쥐의둥지, 쥐의 둥지, 쥐의 보금자리, 쥐의보금자리, 쥐집, 쥐 집, 쥐의집, 쥐의 집</t>
+          <t>리도라, 리들러</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>나조 이름</t>
+          <t>브랜드</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>HIRAMEKI TRUMP</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>히라메키 트럼프, 히라메키트럼프, 히라메키, 트럼프</t>
+          <t>ねずみの巣</t>
+        </is>
+      </c>
+      <c r="C84" s="8" t="inlineStr">
+        <is>
+          <t>쥐의굴, 쥐의 굴, 네즈미노 스, 쥐의둥지, 쥐의 둥지, 쥐의 보금자리, 쥐의보금자리, 쥐집, 쥐 집, 쥐의집, 쥐의 집</t>
         </is>
       </c>
     </row>
@@ -1901,12 +1896,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>HIRAMEKI TRUMP RED</t>
+          <t>HIRAMEKI TRUMP</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>히라메키 트럼프 레드, 히라메키트럼프 레드, 히라메키트럼프레드, 히라메키 트럼프레드, 레드, 히라메키, 트럼프</t>
+          <t>히라메키 트럼프, 히라메키트럼프, 히라메키, 트럼프</t>
         </is>
       </c>
     </row>
@@ -1918,10 +1913,27 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
+          <t>HIRAMEKI TRUMP RED</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>히라메키 트럼프 레드, 히라메키트럼프 레드, 히라메키트럼프레드, 히라메키 트럼프레드, 레드, 히라메키, 트럼프</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>나조 이름</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
           <t>XI</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>일레븐, 엑스아이</t>
         </is>

</xml_diff>